<commit_message>
Use 1600 Livingston Ave as the quote and sample warehouse.
Hope Hill is home — keep it off mill forms. Sphinx and Kash DHL now point at North Brunswick. Glass still prices FOB to NJ; Florida routing can wait.

Co-authored-by: baruchstablet <baruchstablet@gmail.com>
</commit_message>
<xml_diff>
--- a/cursor/product-pricing-analysis/sphinx-glass/Sphinx_Prospect_Registration_AllPro.xlsx
+++ b/cursor/product-pricing-analysis/sphinx-glass/Sphinx_Prospect_Registration_AllPro.xlsx
@@ -119,7 +119,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -141,11 +141,128 @@
         <color rgb="00B0B0B0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -193,6 +310,17 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -597,17 +725,18 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>COMPANY CONTACT</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="22" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -620,7 +749,7 @@
           <t>All Pro Building Supplies LLC</t>
         </is>
       </c>
-      <c r="C6" s="9" t="n"/>
+      <c r="C6" s="22" t="n"/>
       <c r="D6" s="7" t="inlineStr">
         <is>
           <t>COUNTRY</t>
@@ -631,7 +760,7 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="F6" s="9" t="n"/>
+      <c r="F6" s="22" t="n"/>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
@@ -641,11 +770,11 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>35 Hope Hill Lane
-Lakewood, NJ 08701</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="n"/>
+          <t>1600 Livingston Ave
+North Brunswick, NJ 08902</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="n"/>
       <c r="D7" s="7" t="inlineStr">
         <is>
           <t>DISTRICT / STATE</t>
@@ -653,10 +782,10 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>New Jersey (Ocean County / Lakewood)</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="n"/>
+          <t>New Jersey (North Brunswick / Middlesex County)</t>
+        </is>
+      </c>
+      <c r="F7" s="22" t="n"/>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -669,7 +798,7 @@
           <t>Baruch Grossman — Founder &amp; Owner</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n"/>
+      <c r="C8" s="22" t="n"/>
       <c r="D8" s="7" t="inlineStr">
         <is>
           <t>TELEPHONE</t>
@@ -680,7 +809,7 @@
           <t>+1 732-734-1123</t>
         </is>
       </c>
-      <c r="F8" s="9" t="n"/>
+      <c r="F8" s="22" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -693,7 +822,7 @@
           <t>+1 732-734-1123</t>
         </is>
       </c>
-      <c r="C9" s="9" t="n"/>
+      <c r="C9" s="22" t="n"/>
       <c r="D9" s="7" t="inlineStr">
         <is>
           <t>WEBSITE</t>
@@ -704,7 +833,7 @@
           <t>https://allprobuildingsupplies.com</t>
         </is>
       </c>
-      <c r="F9" s="9" t="n"/>
+      <c r="F9" s="22" t="n"/>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -713,7 +842,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr"/>
-      <c r="C10" s="9" t="n"/>
+      <c r="C10" s="22" t="n"/>
       <c r="D10" s="7" t="inlineStr">
         <is>
           <t>CONTACT EMAIL</t>
@@ -725,19 +854,20 @@
 baruch@allprobuildingsupplies.com</t>
         </is>
       </c>
-      <c r="F10" s="9" t="n"/>
-    </row>
+      <c r="F10" s="22" t="n"/>
+    </row>
+    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
           <t>COMPANY OVERVIEW</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
+      <c r="B12" s="21" t="n"/>
+      <c r="C12" s="21" t="n"/>
+      <c r="D12" s="21" t="n"/>
+      <c r="E12" s="21" t="n"/>
+      <c r="F12" s="22" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
@@ -747,29 +877,26 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>US B2B building-supplies importer / wholesaler for contractors and property managers in New Jersey and the East Coast. We sell flooring, plumbing (copper / PVC / CPVC / PEX), and window coverings. We are adding mill-direct annealed clear float glass sheets (windows, storefront, shower, tabletops) — we are NOT a glass processor (no cutting, tempering, or IG). We import FOB origin port into NY/NJ (Newark / Elizabeth). Warehouse is New Jersey. Memphis is a customer job only, not the warehouse.</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="n"/>
-      <c r="D13" s="12" t="n"/>
-      <c r="E13" s="12" t="n"/>
-      <c r="F13" s="12" t="n"/>
+          <t>US B2B building-supplies importer / wholesaler for contractors and property managers in New Jersey and the East Coast. We sell flooring, plumbing (copper / PVC / CPVC / PEX), and window coverings. We are adding mill-direct annealed clear float glass sheets (windows, storefront, shower, tabletops) — we are NOT a glass processor (no cutting, tempering, or IG). We import FOB origin port into NY/NJ (Newark / Elizabeth). Warehouse is 1600 Livingston Ave, North Brunswick, NJ 08902. Memphis and Florida are customer jobs only — still price FOB to NJ first.</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n"/>
+      <c r="D13" s="23" t="n"/>
+      <c r="E13" s="23" t="n"/>
+      <c r="F13" s="24" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="13" t="n"/>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="12" t="n"/>
-      <c r="F14" s="12" t="n"/>
+      <c r="A14" s="25" t="n"/>
+      <c r="B14" s="26" t="n"/>
+      <c r="F14" s="27" t="n"/>
     </row>
     <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="13" t="n"/>
-      <c r="B15" s="12" t="n"/>
-      <c r="C15" s="12" t="n"/>
-      <c r="D15" s="12" t="n"/>
-      <c r="E15" s="12" t="n"/>
-      <c r="F15" s="12" t="n"/>
+      <c r="A15" s="28" t="n"/>
+      <c r="B15" s="29" t="n"/>
+      <c r="C15" s="30" t="n"/>
+      <c r="D15" s="30" t="n"/>
+      <c r="E15" s="30" t="n"/>
+      <c r="F15" s="31" t="n"/>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
@@ -782,7 +909,7 @@
           <t>US importer LLC (Baruch Grossman, Founder). Exact filing year — confirm if you need it; not required for the quote.</t>
         </is>
       </c>
-      <c r="C16" s="9" t="n"/>
+      <c r="C16" s="22" t="n"/>
       <c r="D16" s="7" t="inlineStr">
         <is>
           <t>GROSS ANNUAL CONSUMPTION</t>
@@ -793,7 +920,7 @@
           <t>New glass program. No trailing 12-month glass volume. First PO target: one 20 ft of 6 mm. Then monthly as we sell through. Please quote USD/m² per 20 ft, not a fake monthly run-rate.</t>
         </is>
       </c>
-      <c r="F16" s="9" t="n"/>
+      <c r="F16" s="22" t="n"/>
     </row>
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
@@ -806,7 +933,7 @@
           <t>New Jersey and surrounding US East Coast. Discharge NY/NJ. Do not quote DDP Memphis / Southeast.</t>
         </is>
       </c>
-      <c r="C17" s="9" t="n"/>
+      <c r="C17" s="22" t="n"/>
       <c r="D17" s="7" t="inlineStr">
         <is>
           <t>GLASS SUPPLY SOURCE</t>
@@ -817,7 +944,7 @@
           <t>Seeking mill-direct (Egypt tin-bath). Will not buy China or Malaysia origin (US AD/CVD).</t>
         </is>
       </c>
-      <c r="F17" s="9" t="n"/>
+      <c r="F17" s="22" t="n"/>
     </row>
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
@@ -830,7 +957,7 @@
           <t>Building materials wholesale — contractor / property B2B. Architectural annealed sheet, not auto glass.</t>
         </is>
       </c>
-      <c r="C18" s="9" t="n"/>
+      <c r="C18" s="22" t="n"/>
       <c r="D18" s="7" t="inlineStr">
         <is>
           <t>PROCESSOR / TRADER</t>
@@ -841,19 +968,20 @@
           <t>TRADER / IMPORTER. Not a processor.</t>
         </is>
       </c>
-      <c r="F18" s="9" t="n"/>
-    </row>
+      <c r="F18" s="22" t="n"/>
+    </row>
+    <row r="19"/>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
           <t>SHIPPING INFORMATION</t>
         </is>
       </c>
-      <c r="B20" s="11" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="11" t="n"/>
+      <c r="B20" s="21" t="n"/>
+      <c r="C20" s="21" t="n"/>
+      <c r="D20" s="21" t="n"/>
+      <c r="E20" s="21" t="n"/>
+      <c r="F20" s="22" t="n"/>
     </row>
     <row r="21" ht="40" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
@@ -866,7 +994,7 @@
           <t>FOB Alexandria or Damietta (Egypt load port). FCA same ports OK. NOT EXW factory. NOT DDP USA.</t>
         </is>
       </c>
-      <c r="C21" s="9" t="n"/>
+      <c r="C21" s="22" t="n"/>
       <c r="D21" s="7" t="inlineStr">
         <is>
           <t>EQUIPMENT TYPE</t>
@@ -877,7 +1005,7 @@
           <t>20 ft container, seaworthy A-frame crates / stillages. NOT 40HQ (glass is weight-limited).</t>
         </is>
       </c>
-      <c r="F21" s="9" t="n"/>
+      <c r="F21" s="22" t="n"/>
     </row>
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
@@ -890,7 +1018,7 @@
           <t>Newark / Elizabeth, NJ, USA (NY/NJ)</t>
         </is>
       </c>
-      <c r="C22" s="9" t="n"/>
+      <c r="C22" s="22" t="n"/>
       <c r="D22" s="7" t="inlineStr">
         <is>
           <t>FINAL DESTINATION</t>
@@ -898,22 +1026,23 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>All Pro warehouse, Lakewood, New Jersey, USA (35 Hope Hill Lane, Lakewood NJ 08701). Inland from the port is ours.</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="n"/>
-    </row>
+          <t>All Pro warehouse: 1600 Livingston Ave, North Brunswick, NJ 08902, USA. Inland from Newark/Elizabeth is ours. A Florida job may take a later container direct — still quote FOB + NJ first.</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="n"/>
+    </row>
+    <row r="23"/>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
           <t>PRODUCTS INFORMATION</t>
         </is>
       </c>
-      <c r="B24" s="15" t="n"/>
-      <c r="C24" s="15" t="n"/>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="15" t="n"/>
+      <c r="B24" s="21" t="n"/>
+      <c r="C24" s="21" t="n"/>
+      <c r="D24" s="21" t="n"/>
+      <c r="E24" s="21" t="n"/>
+      <c r="F24" s="22" t="n"/>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="16" t="inlineStr">
@@ -921,7 +1050,7 @@
           <t>PRODUCT NAME</t>
         </is>
       </c>
-      <c r="B25" s="16" t="n"/>
+      <c r="B25" s="22" t="n"/>
       <c r="C25" s="16" t="inlineStr">
         <is>
           <t>QUALITY</t>
@@ -950,7 +1079,7 @@
 — this is the volume SKU</t>
         </is>
       </c>
-      <c r="B26" s="8" t="n"/>
+      <c r="B26" s="22" t="n"/>
       <c r="C26" s="8" t="inlineStr">
         <is>
           <t>Standard commercial clear. EN 572-2 or Sphinx commercial grade. Green edge OK. NOT ultra-clear / low-iron. NOT jumbo unless cheaper per m².</t>
@@ -979,7 +1108,7 @@
           <t>Trulite® Clear Float (annealed)</t>
         </is>
       </c>
-      <c r="B27" s="8" t="n"/>
+      <c r="B27" s="22" t="n"/>
       <c r="C27" s="8" t="inlineStr">
         <is>
           <t>Same commercial clear as 6 mm. Not coated, not tinted.</t>
@@ -1008,7 +1137,7 @@
           <t>Trulite® Clear Float (annealed)</t>
         </is>
       </c>
-      <c r="B28" s="8" t="n"/>
+      <c r="B28" s="22" t="n"/>
       <c r="C28" s="8" t="inlineStr">
         <is>
           <t>Same commercial clear. 12 mm is fine — do NOT quote 12.7 mm true 1/2" at a premium.</t>
@@ -1037,7 +1166,7 @@
           <t>Isolite / SolarLite / Vistalite / jumbo / low-iron / tempered / laminated</t>
         </is>
       </c>
-      <c r="B29" s="17" t="n"/>
+      <c r="B29" s="22" t="n"/>
       <c r="C29" s="17" t="inlineStr">
         <is>
           <t>DO NOT QUOTE</t>
@@ -1067,17 +1196,18 @@
       </c>
     </row>
     <row r="31" ht="22" customHeight="1"/>
+    <row r="32"/>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
           <t>NAME / SIGNATURE</t>
         </is>
       </c>
-      <c r="B33" s="6" t="n"/>
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="6" t="n"/>
-      <c r="E33" s="6" t="n"/>
-      <c r="F33" s="6" t="n"/>
+      <c r="B33" s="21" t="n"/>
+      <c r="C33" s="21" t="n"/>
+      <c r="D33" s="21" t="n"/>
+      <c r="E33" s="21" t="n"/>
+      <c r="F33" s="22" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -1090,7 +1220,7 @@
           <t>Baruch Grossman</t>
         </is>
       </c>
-      <c r="C34" s="9" t="n"/>
+      <c r="C34" s="22" t="n"/>
       <c r="D34" s="7" t="inlineStr">
         <is>
           <t>TITLE</t>
@@ -1101,7 +1231,7 @@
           <t>Founder &amp; Owner</t>
         </is>
       </c>
-      <c r="F34" s="9" t="n"/>
+      <c r="F34" s="22" t="n"/>
     </row>
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="7" t="inlineStr">
@@ -1114,7 +1244,7 @@
           <t>(please sign here before sending)</t>
         </is>
       </c>
-      <c r="C35" s="9" t="n"/>
+      <c r="C35" s="22" t="n"/>
       <c r="D35" s="7" t="inlineStr">
         <is>
           <t>DATE</t>
@@ -1125,7 +1255,7 @@
           <t>7 September 2026</t>
         </is>
       </c>
-      <c r="F35" s="9" t="n"/>
+      <c r="F35" s="22" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="41">
@@ -1236,7 +1366,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>35 Hope Hill Lane, Lakewood, NJ 08701, USA</t>
+          <t>1600 Livingston Ave, North Brunswick, NJ 08902, USA</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1582,7 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>All Pro warehouse, Lakewood NJ 08701 (inland from port is ours)</t>
+          <t>1600 Livingston Ave, North Brunswick, NJ 08902 (inland from port is ours)</t>
         </is>
       </c>
     </row>
@@ -1711,6 +1841,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="420" customHeight="1">
       <c r="A3" s="20" t="inlineStr">
         <is>
@@ -1723,7 +1854,7 @@
 • Stock sheet sizes you already cut (2140×3210, 2250×3210, 1830×2440, or closest). Jumbo only if cheaper per m².
 • Packing: 20 ft A-frame crates (not 40HQ).
 • Incoterm: FOB Alexandria or Damietta. Not EXW, not DDP.
-• Discharge: Newark / Elizabeth, NJ, USA. Final warehouse is New Jersey (not Memphis).
+• Discharge: Newark / Elizabeth, NJ, USA. Final warehouse is 1600 Livingston Ave, North Brunswick, NJ 08902. A Florida customer may take a later load direct — still quote FOB + NJ first (not Memphis, not DDP Florida).
 Need back: USD/m² FOB, kg/m², m² per 20 ft, crate count, MOQ, lead time, and confirmation the tin-bath is Egypt.
 First order target is one 20 ft of 6 mm. 10 mm and 12 mm are for pricing so we can add them after 6 mm sells.
 Best regards,

</xml_diff>